<commit_message>
Add generation-length and GC sensitivity analyses
Generation length from Bird et al. (2020) for the 84 taxa (13b), written
into Table S2 of Table_S1.xlsx (14c), with the great auk's extrapolated
value and its missing genome GC imputed by phylo.impute in script 14,
which also fixes the GC lookup for Feng's trinomial names.

Opt-in sensitivity modes with suffixed outputs: SENS=gen and SENS=gc in
scripts 16, 16b and 16c (generation length in place of body mass, GC as a
fourth response), MRPMM_COVAR=gen in script 23 (generation length as a
fixed effect), and GC3=TRUE in script 20b using per-gene GC3 from 19b.

Script 23 runs on GenomeDK without phytools, and combines its priors in a
way that brms 2.22 accepts. Job scripts in hpc/brms and hpc/impute.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Table_S1.xlsx
+++ b/data/Table_S1.xlsx
@@ -7908,6 +7908,16 @@
           <t xml:space="preserve">Morphometric source</t>
         </is>
       </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Generation length (years)</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Generation length source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8043,6 +8053,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS2">
+        <v>9.2552</v>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8178,6 +8196,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS3">
+        <v>4.6842</v>
+      </c>
+      <c r="AT3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8323,6 +8349,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS4">
+        <v>8.2979</v>
+      </c>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8473,6 +8507,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS5">
+        <v>4.7810</v>
+      </c>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8632,6 +8674,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS6">
+        <v>4.6898</v>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8777,6 +8827,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS7">
+        <v>2.6339</v>
+      </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -8922,6 +8980,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS8">
+        <v>5.2826</v>
+      </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -9072,6 +9138,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS9">
+        <v>2.1668</v>
+      </c>
+      <c r="AT9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9227,6 +9301,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS10">
+        <v>3.4283</v>
+      </c>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -9382,6 +9464,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS11">
+        <v>5.4486</v>
+      </c>
+      <c r="AT11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9527,6 +9617,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS12">
+        <v>4.7872</v>
+      </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -9677,6 +9775,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS13">
+        <v>4.1856</v>
+      </c>
+      <c r="AT13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9822,6 +9928,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS14">
+        <v>7.6027</v>
+      </c>
+      <c r="AT14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -9972,6 +10086,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS15">
+        <v>5.3958</v>
+      </c>
+      <c r="AT15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -10117,6 +10239,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS16">
+        <v>3.2167</v>
+      </c>
+      <c r="AT16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -10267,6 +10397,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS17">
+        <v>3.1924</v>
+      </c>
+      <c r="AT17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -10412,6 +10550,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS18">
+        <v>3.3741</v>
+      </c>
+      <c r="AT18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -10562,6 +10708,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS19">
+        <v>2.7565</v>
+      </c>
+      <c r="AT19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -10697,6 +10851,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS20">
+        <v>5.2123</v>
+      </c>
+      <c r="AT20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -10837,6 +10999,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS21">
+        <v>3.8642</v>
+      </c>
+      <c r="AT21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -10982,6 +11152,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS22">
+        <v>3.9931</v>
+      </c>
+      <c r="AT22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -11132,6 +11310,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS23">
+        <v>4.3941</v>
+      </c>
+      <c r="AT23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -11272,6 +11458,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS24">
+        <v>6.4802</v>
+      </c>
+      <c r="AT24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -11412,6 +11606,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS25">
+        <v>9.2522</v>
+      </c>
+      <c r="AT25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -11552,6 +11754,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS26">
+        <v>3.6876</v>
+      </c>
+      <c r="AT26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -11697,6 +11907,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS27">
+        <v>4.5417</v>
+      </c>
+      <c r="AT27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -11861,6 +12079,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS28">
+        <v>3.9240</v>
+      </c>
+      <c r="AT28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -12016,6 +12242,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS29">
+        <v>4.0580</v>
+      </c>
+      <c r="AT29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -12149,6 +12383,14 @@
           <t xml:space="preserve">Livezey 1988 Table 1 (morphometrics); Montgomerie &amp; Birkhead 2025 (mass)</t>
         </is>
       </c>
+      <c r="AS30">
+        <v>23.6879</v>
+      </c>
+      <c r="AT30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Imputed with phylo.impute from ln body mass (Bird et al. 2020 value is a family-level extrapolation)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -12318,6 +12560,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS31">
+        <v>16.3696</v>
+      </c>
+      <c r="AT31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -12453,6 +12703,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS32">
+        <v>7.6049</v>
+      </c>
+      <c r="AT32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -12593,6 +12851,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS33">
+        <v>8.1684</v>
+      </c>
+      <c r="AT33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -12733,6 +12999,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS34">
+        <v>16.4015</v>
+      </c>
+      <c r="AT34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -12878,6 +13152,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS35">
+        <v>7.1015</v>
+      </c>
+      <c r="AT35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -13028,6 +13310,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS36">
+        <v>7.3826</v>
+      </c>
+      <c r="AT36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -13183,6 +13473,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS37">
+        <v>8.7106</v>
+      </c>
+      <c r="AT37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -13328,6 +13626,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS38">
+        <v>5.7600</v>
+      </c>
+      <c r="AT38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -13478,6 +13784,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS39">
+        <v>7.3888</v>
+      </c>
+      <c r="AT39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -13618,6 +13932,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS40">
+        <v>4.4877</v>
+      </c>
+      <c r="AT40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -13768,6 +14090,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS41">
+        <v>13.2360</v>
+      </c>
+      <c r="AT41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -13913,6 +14243,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS42">
+        <v>5.7420</v>
+      </c>
+      <c r="AT42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -14063,6 +14401,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS43">
+        <v>4.2432</v>
+      </c>
+      <c r="AT43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -14213,6 +14559,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS44">
+        <v>3.3614</v>
+      </c>
+      <c r="AT44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -14363,6 +14717,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS45">
+        <v>4.0557</v>
+      </c>
+      <c r="AT45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -14508,6 +14870,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS46">
+        <v>2.5461</v>
+      </c>
+      <c r="AT46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -14672,6 +15042,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS47">
+        <v>3.0094</v>
+      </c>
+      <c r="AT47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -14817,6 +15195,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS48">
+        <v>2.3688</v>
+      </c>
+      <c r="AT48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -14967,6 +15353,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS49">
+        <v>2.0797</v>
+      </c>
+      <c r="AT49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -15121,6 +15515,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS50">
+        <v>5.8159</v>
+      </c>
+      <c r="AT50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -15261,6 +15663,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS51">
+        <v>6.6523</v>
+      </c>
+      <c r="AT51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -15411,6 +15821,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS52">
+        <v>14.4512</v>
+      </c>
+      <c r="AT52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -15575,6 +15993,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS53">
+        <v>16.2553</v>
+      </c>
+      <c r="AT53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -15720,6 +16146,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS54">
+        <v>3.4379</v>
+      </c>
+      <c r="AT54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -15865,6 +16299,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS55">
+        <v>2.5338</v>
+      </c>
+      <c r="AT55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -16010,6 +16452,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS56">
+        <v>3.6494</v>
+      </c>
+      <c r="AT56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -16155,6 +16605,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS57">
+        <v>4.0218</v>
+      </c>
+      <c r="AT57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -16295,6 +16753,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS58">
+        <v>11.8055</v>
+      </c>
+      <c r="AT58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -16435,6 +16901,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS59">
+        <v>19.2924</v>
+      </c>
+      <c r="AT59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -16575,6 +17049,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS60">
+        <v>4.0451</v>
+      </c>
+      <c r="AT60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -16720,6 +17202,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS61">
+        <v>3.3796</v>
+      </c>
+      <c r="AT61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -16874,6 +17364,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS62">
+        <v>2.5345</v>
+      </c>
+      <c r="AT62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -17014,6 +17512,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS63">
+        <v>3.0833</v>
+      </c>
+      <c r="AT63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -17159,6 +17665,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS64">
+        <v>7.5756</v>
+      </c>
+      <c r="AT64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -17304,6 +17818,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS65">
+        <v>8.3172</v>
+      </c>
+      <c r="AT65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -17449,6 +17971,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS66">
+        <v>7.1059</v>
+      </c>
+      <c r="AT66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -17599,6 +18129,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS67">
+        <v>5.7124</v>
+      </c>
+      <c r="AT67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -17739,6 +18277,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS68">
+        <v>7.8762</v>
+      </c>
+      <c r="AT68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -17884,6 +18430,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS69">
+        <v>3.8522</v>
+      </c>
+      <c r="AT69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -18029,6 +18583,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS70">
+        <v>3.6265</v>
+      </c>
+      <c r="AT70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -18174,6 +18736,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS71">
+        <v>2.1999</v>
+      </c>
+      <c r="AT71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -18314,6 +18884,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS72">
+        <v>3.0160</v>
+      </c>
+      <c r="AT72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -18454,6 +19032,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS73">
+        <v>3.0021</v>
+      </c>
+      <c r="AT73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -18594,6 +19180,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS74">
+        <v>4.3141</v>
+      </c>
+      <c r="AT74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -18734,6 +19328,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS75">
+        <v>12.6722</v>
+      </c>
+      <c r="AT75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -18874,6 +19476,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS76">
+        <v>5.8123</v>
+      </c>
+      <c r="AT76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -19014,6 +19624,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS77">
+        <v>3.4338</v>
+      </c>
+      <c r="AT77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -19159,6 +19777,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS78">
+        <v>5.1755</v>
+      </c>
+      <c r="AT78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -19309,6 +19935,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS79">
+        <v>7.9936</v>
+      </c>
+      <c r="AT79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -19454,6 +20088,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS80">
+        <v>2.1425</v>
+      </c>
+      <c r="AT80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -19604,6 +20246,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS81">
+        <v>2.0553</v>
+      </c>
+      <c r="AT81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -19749,6 +20399,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS82">
+        <v>2.1443</v>
+      </c>
+      <c r="AT82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -19899,6 +20557,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS83">
+        <v>1.5705</v>
+      </c>
+      <c r="AT83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -20044,6 +20710,14 @@
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
         </is>
       </c>
+      <c r="AS84">
+        <v>3.0740</v>
+      </c>
+      <c r="AT84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -20187,6 +20861,14 @@
       <c r="AR85" t="inlineStr">
         <is>
           <t xml:space="preserve">AVONET (Tobias et al. 2022)</t>
+        </is>
+      </c>
+      <c r="AS85">
+        <v>2.7988</v>
+      </c>
+      <c r="AT85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bird et al. 2020, Table S4</t>
         </is>
       </c>
     </row>

</xml_diff>